<commit_message>
Preparing VISSIM Session 2 2026 A
</commit_message>
<xml_diff>
--- a/Tools/Signal_Timing_2025.xlsx
+++ b/Tools/Signal_Timing_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iisak\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEVE\vissim_exe\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7304AD15-364B-41A6-A3C3-8A6010BA6675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CE3839-1E06-4A36-AC6A-75835C4EDAA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="18696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-34665" yWindow="2040" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -410,23 +410,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.33203125" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" customWidth="1"/>
-    <col min="3" max="3" width="12.88671875" customWidth="1"/>
-    <col min="4" max="4" width="10.77734375" customWidth="1"/>
-    <col min="5" max="5" width="12.109375" customWidth="1"/>
-    <col min="6" max="6" width="16.21875" customWidth="1"/>
-    <col min="7" max="7" width="14.21875" customWidth="1"/>
+    <col min="1" max="1" width="21.28515625" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -449,75 +449,84 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
+      <c r="B4">
+        <v>600</v>
+      </c>
       <c r="C4">
         <v>1800</v>
       </c>
       <c r="D4" s="2">
         <f>B4/C4</f>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="E4">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F4" s="3">
         <f>(1.5*E4+5)/(1-D7)</f>
-        <v>18.5</v>
-      </c>
-      <c r="G4" s="3" t="e">
+        <v>65.999999999999986</v>
+      </c>
+      <c r="G4" s="3">
         <f>(F4-E4)*D4/D7</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>29.142857142857135</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
+      <c r="B5">
+        <v>150</v>
+      </c>
       <c r="C5">
         <v>1800</v>
       </c>
       <c r="D5" s="2">
         <f t="shared" ref="D5:D6" si="0">B5/C5</f>
-        <v>0</v>
-      </c>
-      <c r="G5" s="3" t="e">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="G5" s="3">
         <f>(F4-E4)*D5/D7</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>7.2857142857142838</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
+      <c r="B6">
+        <v>300</v>
+      </c>
       <c r="C6">
         <v>1800</v>
       </c>
       <c r="D6" s="2">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G6" s="3" t="e">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="G6" s="3">
         <f>(F4-E4)*D6/D7</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>14.571428571428568</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="2">
         <f>SUM(D4:D6)</f>
-        <v>0</v>
-      </c>
-      <c r="G7" s="3" t="e">
+        <v>0.58333333333333326</v>
+      </c>
+      <c r="G7" s="3">
         <f>SUM(G4:G6)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>50.999999999999986</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -540,7 +549,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>1</v>
       </c>
@@ -552,18 +561,18 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F11" s="3">
         <f>(1.5*E11+5)/(1-D14)</f>
-        <v>18.5</v>
+        <v>27.5</v>
       </c>
       <c r="G11" s="3" t="e">
         <f>(F11-E11)*D11/D14</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -579,7 +588,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -595,7 +604,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
Sim2 group3 quecount outputs
</commit_message>
<xml_diff>
--- a/Tools/Signal_Timing_2025.xlsx
+++ b/Tools/Signal_Timing_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEVE\vissim_exe\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CE3839-1E06-4A36-AC6A-75835C4EDAA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E67C28C-BAA0-4FDD-90CC-EB7D1186880E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-34665" yWindow="2040" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -453,64 +453,55 @@
       <c r="A4" t="s">
         <v>1</v>
       </c>
-      <c r="B4">
-        <v>600</v>
-      </c>
       <c r="C4">
         <v>1800</v>
       </c>
       <c r="D4" s="2">
         <f>B4/C4</f>
-        <v>0.33333333333333331</v>
+        <v>0</v>
       </c>
       <c r="E4">
         <v>15</v>
       </c>
       <c r="F4" s="3">
         <f>(1.5*E4+5)/(1-D7)</f>
-        <v>65.999999999999986</v>
-      </c>
-      <c r="G4" s="3">
+        <v>27.5</v>
+      </c>
+      <c r="G4" s="3" t="e">
         <f>(F4-E4)*D4/D7</f>
-        <v>29.142857142857135</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B5">
-        <v>150</v>
-      </c>
       <c r="C5">
         <v>1800</v>
       </c>
       <c r="D5" s="2">
         <f t="shared" ref="D5:D6" si="0">B5/C5</f>
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="G5" s="3">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="e">
         <f>(F4-E4)*D5/D7</f>
-        <v>7.2857142857142838</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
-      <c r="B6">
-        <v>300</v>
-      </c>
       <c r="C6">
         <v>1800</v>
       </c>
       <c r="D6" s="2">
         <f t="shared" si="0"/>
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="G6" s="3">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="e">
         <f>(F4-E4)*D6/D7</f>
-        <v>14.571428571428568</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -519,11 +510,11 @@
       </c>
       <c r="D7" s="2">
         <f>SUM(D4:D6)</f>
-        <v>0.58333333333333326</v>
-      </c>
-      <c r="G7" s="3">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3" t="e">
         <f>SUM(G4:G6)</f>
-        <v>50.999999999999986</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>